<commit_message>
optimizacion de la actualizacion de la base de datos. tambien se creo un archivo config.py
</commit_message>
<xml_diff>
--- a/LISTAS/BISAGRA ALACENA.xlsx
+++ b/LISTAS/BISAGRA ALACENA.xlsx
@@ -861,14 +861,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="27" t="n">
-        <v>45163.60818223692</v>
+        <v>45163.60818223379</v>
       </c>
       <c r="E1" s="4" t="n"/>
     </row>
-    <row r="2"/>
-    <row r="3"/>
-    <row r="4"/>
-    <row r="5"/>
     <row r="6" ht="22.5" customHeight="1" s="17">
       <c r="A6" s="2" t="inlineStr">
         <is>
@@ -920,16 +916,6 @@
       <c r="C12" s="38" t="n"/>
       <c r="D12" s="38" t="n"/>
     </row>
-    <row r="13"/>
-    <row r="14"/>
-    <row r="15"/>
-    <row r="16"/>
-    <row r="17"/>
-    <row r="18"/>
-    <row r="19"/>
-    <row r="20"/>
-    <row r="21"/>
-    <row r="22"/>
     <row r="23">
       <c r="C23" s="19" t="n"/>
     </row>
@@ -985,7 +971,7 @@
       </c>
       <c r="C29" s="39" t="n"/>
       <c r="D29" s="40" t="n">
-        <v>229.739</v>
+        <v>113.89</v>
       </c>
     </row>
     <row r="30" ht="19.5" customHeight="1" s="17">
@@ -1001,15 +987,12 @@
       </c>
       <c r="C30" s="39" t="n"/>
       <c r="D30" s="40" t="n">
-        <v>155.852</v>
+        <v>77.26000000000001</v>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="17">
       <c r="D31" s="41" t="n"/>
     </row>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
     <row r="35" ht="18" customHeight="1" s="17">
       <c r="A35" s="29" t="n"/>
       <c r="B35" s="29" t="n"/>
@@ -1029,34 +1012,30 @@
     <row r="39" ht="19.5" customHeight="1" s="17">
       <c r="B39" s="30" t="n"/>
     </row>
-    <row r="40"/>
-    <row r="41"/>
     <row r="42" ht="19.5" customHeight="1" s="17">
       <c r="A42" s="7" t="n"/>
     </row>
-    <row r="43"/>
     <row r="44">
       <c r="A44" s="5" t="n"/>
     </row>
-    <row r="45"/>
     <row r="46">
       <c r="A46" s="6" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="13">
     <mergeCell ref="B39:C39"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="A12:D12"/>
     <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A9:D9"/>
+    <mergeCell ref="B28:C28"/>
+    <mergeCell ref="B36:C36"/>
+    <mergeCell ref="A11:D11"/>
+    <mergeCell ref="A10:D10"/>
     <mergeCell ref="B35:C35"/>
-    <mergeCell ref="B36:C36"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A11:D11"/>
-    <mergeCell ref="B28:C28"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B30:C30"/>
-    <mergeCell ref="A12:D12"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0" footer="0"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>